<commit_message>
Mise à jour du livrable (build 2026-09-09) — assurance vie & épargne-pension
</commit_message>
<xml_diff>
--- a/Exemple-import.xlsx
+++ b/Exemple-import.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -442,6 +442,7 @@
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,6 +526,11 @@
           <t>Région</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Versement annuel</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -904,6 +910,88 @@
         <is>
           <t>Belgique</t>
         </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Assurance vie (branche 21)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Assurance vie</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>15000</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>AG Insurance</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>capital garanti, exonéré après 8 ans</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Belgique</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Épargne-pension</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Épargne-pension</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>KBC</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>réduction d'impôt à l'entrée, taxe à 60 ans</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Belgique</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>1020</v>
       </c>
     </row>
   </sheetData>

</xml_diff>